<commit_message>
Separate year and property ID columns visually in the sample workbook
</commit_message>
<xml_diff>
--- a/state-project/inputs/state-practice.xlsx
+++ b/state-project/inputs/state-practice.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Book" sheetId="1" r:id="Rc4466c4966f942a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bill" sheetId="2" r:id="R8328aec836474c4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Book" sheetId="1" r:id="R8c06f345f71e4278"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bill" sheetId="2" r:id="R0c7b1a0d775e4584"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -65,13 +65,18 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -318,13 +323,13 @@
       <x:c r="A4" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C4" s="6" t="str">
+      <x:c r="B4" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
         <x:v>001101</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="n">
+      <x:c r="D4" s="8" t="n">
         <x:v>100</x:v>
       </x:c>
     </x:row>
@@ -332,13 +337,13 @@
       <x:c r="A5" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="str">
+      <x:c r="B5" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="str">
         <x:v>001102</x:v>
       </x:c>
-      <x:c r="D5" s="7" t="n">
+      <x:c r="D5" s="8" t="n">
         <x:v>200</x:v>
       </x:c>
     </x:row>
@@ -346,13 +351,13 @@
       <x:c r="A6" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="str">
+      <x:c r="B6" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="str">
         <x:v>001103</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="n">
+      <x:c r="D6" s="8" t="n">
         <x:v>300</x:v>
       </x:c>
     </x:row>
@@ -360,13 +365,13 @@
       <x:c r="A7" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="str">
+      <x:c r="B7" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="str">
         <x:v>001104</x:v>
       </x:c>
-      <x:c r="D7" s="7" t="n">
+      <x:c r="D7" s="8" t="n">
         <x:v>400</x:v>
       </x:c>
     </x:row>
@@ -374,15 +379,15 @@
       <x:c r="A8" s="1"/>
       <x:c r="B8" s="1"/>
       <x:c r="C8" s="1"/>
-      <x:c r="D8" s="7"/>
+      <x:c r="D8" s="8"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="8" t="str">
+      <x:c r="A9" s="9" t="str">
         <x:v>Control total</x:v>
       </x:c>
-      <x:c r="B9" s="8"/>
-      <x:c r="C9" s="8"/>
-      <x:c r="D9" s="9" t="n">
+      <x:c r="B9" s="9"/>
+      <x:c r="C9" s="9"/>
+      <x:c r="D9" s="10" t="n">
         <x:f>SUM(D4:D7)</x:f>
         <x:v>1000</x:v>
       </x:c>
@@ -450,13 +455,13 @@
       <x:c r="A4" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C4" s="6" t="str">
+      <x:c r="B4" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
         <x:v>001101</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="n">
+      <x:c r="D4" s="8" t="n">
         <x:v>100</x:v>
       </x:c>
     </x:row>
@@ -464,13 +469,13 @@
       <x:c r="A5" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="str">
+      <x:c r="B5" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C5" s="7" t="str">
         <x:v>001102</x:v>
       </x:c>
-      <x:c r="D5" s="7" t="n">
+      <x:c r="D5" s="8" t="n">
         <x:v>210</x:v>
       </x:c>
     </x:row>
@@ -478,13 +483,13 @@
       <x:c r="A6" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="str">
+      <x:c r="B6" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="str">
         <x:v>001103</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="n">
+      <x:c r="D6" s="8" t="n">
         <x:v>290</x:v>
       </x:c>
     </x:row>
@@ -492,13 +497,13 @@
       <x:c r="A7" s="1" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="n">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="str">
+      <x:c r="B7" s="6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="str">
         <x:v>001105</x:v>
       </x:c>
-      <x:c r="D7" s="7" t="n">
+      <x:c r="D7" s="8" t="n">
         <x:v>500</x:v>
       </x:c>
     </x:row>
@@ -506,15 +511,15 @@
       <x:c r="A8" s="1"/>
       <x:c r="B8" s="1"/>
       <x:c r="C8" s="1"/>
-      <x:c r="D8" s="7"/>
+      <x:c r="D8" s="8"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="8" t="str">
+      <x:c r="A9" s="9" t="str">
         <x:v>Control total</x:v>
       </x:c>
-      <x:c r="B9" s="8"/>
-      <x:c r="C9" s="8"/>
-      <x:c r="D9" s="9" t="n">
+      <x:c r="B9" s="9"/>
+      <x:c r="C9" s="9"/>
+      <x:c r="D9" s="10" t="n">
         <x:f>SUM(D4:D7)</x:f>
         <x:v>1100</x:v>
       </x:c>

</xml_diff>